<commit_message>
Removed the REINFORCE-like term of the entropy for the gradient calcualtions. Implemented the temperature for the structure head (not tested enough yet). Added logging for rendering time. Added a new application for RPA with larger networks (seemed to work). Added init files.
</commit_message>
<xml_diff>
--- a/apps_MAK_REINFORCE/multistability_2species_6rxns/multistability_2species_6rxns_MAK_REINFORCE.xlsx
+++ b/apps_MAK_REINFORCE/multistability_2species_6rxns/multistability_2species_6rxns_MAK_REINFORCE.xlsx
@@ -204,7 +204,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -215,12 +215,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -252,15 +246,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="8">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
@@ -269,13 +260,7 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -283,9 +268,6 @@
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -592,15 +574,15 @@
   <dimension ref="A1:I27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="34.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="10" width="19.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="10" width="20.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="10" width="22.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="10" width="24.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="34.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="19.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="20.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="22.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="24.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -628,7 +610,7 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -657,7 +639,7 @@
       <c r="H2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -665,28 +647,28 @@
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>6</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>6</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>6</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>6</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="3">
         <v>6</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="3">
         <v>6</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="3">
         <v>6</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="3">
         <v>6</v>
       </c>
     </row>
@@ -694,28 +676,28 @@
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>2</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>2</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>2</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>2</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>2</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="3">
         <v>2</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="3">
         <v>2</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="3">
         <v>2</v>
       </c>
     </row>
@@ -723,28 +705,28 @@
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="4">
-        <v>1</v>
-      </c>
-      <c r="C5" s="4">
-        <v>1</v>
-      </c>
-      <c r="D5" s="4">
-        <v>1</v>
-      </c>
-      <c r="E5" s="4">
-        <v>1</v>
-      </c>
-      <c r="F5" s="4">
-        <v>1</v>
-      </c>
-      <c r="G5" s="4">
-        <v>1</v>
-      </c>
-      <c r="H5" s="4">
-        <v>1</v>
-      </c>
-      <c r="I5" s="4">
+      <c r="B5" s="3">
+        <v>1</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
+      <c r="G5" s="3">
+        <v>1</v>
+      </c>
+      <c r="H5" s="3">
+        <v>1</v>
+      </c>
+      <c r="I5" s="3">
         <v>1</v>
       </c>
     </row>
@@ -752,28 +734,28 @@
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>1280</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="3">
         <v>1280</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>1280</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>1280</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="3">
         <v>1280</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="3">
         <v>1280</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="3">
         <v>1280</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="3">
         <v>1280</v>
       </c>
     </row>
@@ -781,28 +763,28 @@
       <c r="A7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="5" t="b">
+      <c r="B7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="C7" s="5" t="b">
+      <c r="C7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="D7" s="5" t="b">
+      <c r="D7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="5" t="b">
+      <c r="E7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="F7" s="5" t="b">
+      <c r="F7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G7" s="5" t="b">
+      <c r="G7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H7" s="5" t="b">
+      <c r="H7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="I7" s="6" t="b">
+      <c r="I7" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -810,28 +792,28 @@
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="5">
         <v>0.00005</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="5">
         <v>0.00003</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="5">
         <v>0.00001</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="5">
         <v>0.00001</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="5">
         <v>0.00001</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="5">
         <v>0.0001</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="5">
         <v>0.0001</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="5">
         <v>0.00002</v>
       </c>
     </row>
@@ -839,28 +821,28 @@
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="3">
         <v>400</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="3">
         <v>300</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="3">
         <v>400</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <v>400</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="3">
         <v>700</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="3">
         <v>400</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="3">
         <v>400</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="3">
         <v>400</v>
       </c>
     </row>
@@ -868,28 +850,28 @@
       <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="3">
         <v>5</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="3">
         <v>5</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>5</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <v>5</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="3">
         <v>5</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="3">
         <v>5</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="3">
         <v>5</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="3">
         <v>5</v>
       </c>
     </row>
@@ -897,28 +879,28 @@
       <c r="A11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="3">
         <v>1024</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="3">
         <v>1024</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="3">
         <v>1024</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <v>1024</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="3">
         <v>1024</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="3">
         <v>1024</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="3">
         <v>1024</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I11" s="3">
         <v>1024</v>
       </c>
     </row>
@@ -926,28 +908,28 @@
       <c r="A12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="3">
         <v>10240</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="3">
         <v>10240</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="3">
         <v>10240</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="3">
         <v>10240</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="3">
         <v>10240</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="3">
         <v>10240</v>
       </c>
-      <c r="H12" s="4">
+      <c r="H12" s="3">
         <v>10240</v>
       </c>
-      <c r="I12" s="4">
+      <c r="I12" s="3">
         <v>10240</v>
       </c>
     </row>
@@ -955,28 +937,28 @@
       <c r="A13" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="3">
         <v>128</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="3">
         <v>128</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="3">
         <v>128</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="3">
         <v>128</v>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="3">
         <v>128</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="3">
         <v>128</v>
       </c>
-      <c r="H13" s="4">
+      <c r="H13" s="3">
         <v>128</v>
       </c>
-      <c r="I13" s="4">
+      <c r="I13" s="3">
         <v>128</v>
       </c>
     </row>
@@ -1005,7 +987,7 @@
       <c r="H14" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1034,7 +1016,7 @@
       <c r="H15" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="I15" s="2" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1042,28 +1024,28 @@
       <c r="A16" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B16" s="4">
-        <v>1</v>
-      </c>
-      <c r="C16" s="4">
-        <v>1</v>
-      </c>
-      <c r="D16" s="4">
-        <v>1</v>
-      </c>
-      <c r="E16" s="4">
-        <v>1</v>
-      </c>
-      <c r="F16" s="4">
-        <v>1</v>
-      </c>
-      <c r="G16" s="4">
-        <v>1</v>
-      </c>
-      <c r="H16" s="4">
-        <v>1</v>
-      </c>
-      <c r="I16" s="4">
+      <c r="B16" s="3">
+        <v>1</v>
+      </c>
+      <c r="C16" s="3">
+        <v>1</v>
+      </c>
+      <c r="D16" s="3">
+        <v>1</v>
+      </c>
+      <c r="E16" s="3">
+        <v>1</v>
+      </c>
+      <c r="F16" s="3">
+        <v>1</v>
+      </c>
+      <c r="G16" s="3">
+        <v>1</v>
+      </c>
+      <c r="H16" s="3">
+        <v>1</v>
+      </c>
+      <c r="I16" s="3">
         <v>1</v>
       </c>
     </row>
@@ -1071,28 +1053,28 @@
       <c r="A17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="3">
         <v>20</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="3">
         <v>20</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="3">
         <v>20</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="3">
         <v>20</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="3">
         <v>20</v>
       </c>
-      <c r="G17" s="4">
+      <c r="G17" s="3">
         <v>20</v>
       </c>
-      <c r="H17" s="4">
+      <c r="H17" s="3">
         <v>20</v>
       </c>
-      <c r="I17" s="4">
+      <c r="I17" s="3">
         <v>20</v>
       </c>
     </row>
@@ -1100,28 +1082,28 @@
       <c r="A18" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="3">
         <v>100</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="3">
         <v>100</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="3">
         <v>100</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="3">
         <v>100</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="3">
         <v>100</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18" s="3">
         <v>100</v>
       </c>
-      <c r="H18" s="4">
+      <c r="H18" s="3">
         <v>100</v>
       </c>
-      <c r="I18" s="4">
+      <c r="I18" s="3">
         <v>100</v>
       </c>
     </row>
@@ -1129,28 +1111,28 @@
       <c r="A19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="3">
         <v>1000</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="3">
         <v>1000</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="3">
         <v>1000</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="3">
         <v>1000</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="3">
         <v>1000</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19" s="3">
         <v>1000</v>
       </c>
-      <c r="H19" s="4">
+      <c r="H19" s="3">
         <v>1000</v>
       </c>
-      <c r="I19" s="4">
+      <c r="I19" s="3">
         <v>1000</v>
       </c>
     </row>
@@ -1158,28 +1140,28 @@
       <c r="A20" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="3">
         <v>32</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C20" s="3">
         <v>32</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="3">
         <v>32</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="3">
         <v>32</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="3">
         <v>32</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G20" s="3">
         <v>32</v>
       </c>
-      <c r="H20" s="4">
+      <c r="H20" s="3">
         <v>32</v>
       </c>
-      <c r="I20" s="4">
+      <c r="I20" s="3">
         <v>32</v>
       </c>
     </row>
@@ -1187,28 +1169,28 @@
       <c r="A21" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="4">
-        <v>1</v>
-      </c>
-      <c r="C21" s="4">
-        <v>1</v>
-      </c>
-      <c r="D21" s="4">
-        <v>1</v>
-      </c>
-      <c r="E21" s="4">
-        <v>1</v>
-      </c>
-      <c r="F21" s="4">
-        <v>1</v>
-      </c>
-      <c r="G21" s="4">
-        <v>1</v>
-      </c>
-      <c r="H21" s="4">
-        <v>1</v>
-      </c>
-      <c r="I21" s="4">
+      <c r="B21" s="3">
+        <v>1</v>
+      </c>
+      <c r="C21" s="3">
+        <v>1</v>
+      </c>
+      <c r="D21" s="3">
+        <v>1</v>
+      </c>
+      <c r="E21" s="3">
+        <v>1</v>
+      </c>
+      <c r="F21" s="3">
+        <v>1</v>
+      </c>
+      <c r="G21" s="3">
+        <v>1</v>
+      </c>
+      <c r="H21" s="3">
+        <v>1</v>
+      </c>
+      <c r="I21" s="3">
         <v>1</v>
       </c>
     </row>
@@ -1237,7 +1219,7 @@
       <c r="H22" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="I22" s="3" t="s">
+      <c r="I22" s="2" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1248,25 +1230,25 @@
       <c r="B23" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="I23" s="8" t="s">
+      <c r="C23" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I23" s="3" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1277,25 +1259,25 @@
       <c r="B24" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F24" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G24" s="4" t="s">
+      <c r="F24" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G24" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="H24" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="I24" s="8" t="s">
+      <c r="I24" s="3" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1312,19 +1294,19 @@
       <c r="D25" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H25" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="I25" s="8" t="s">
+      <c r="E25" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I25" s="3" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1335,25 +1317,25 @@
       <c r="B26" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="C26" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E26" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H26" s="4" t="s">
+      <c r="E26" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H26" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="I26" s="8" t="s">
+      <c r="I26" s="3" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1382,7 +1364,7 @@
       <c r="H27" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="I27" s="3" t="s">
+      <c r="I27" s="2" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>